<commit_message>
Sensibilidades con el modelo verificado: script de supuestos y hojas regeneradas
</commit_message>
<xml_diff>
--- a/sensibilidad_cortocircuito.xlsx
+++ b/sensibilidad_cortocircuito.xlsx
@@ -411,13 +411,13 @@
         <v>500</v>
       </c>
       <c r="B2">
-        <v>6.5</v>
+        <v>6.81</v>
       </c>
       <c r="C2">
-        <v>4.516</v>
+        <v>8.128</v>
       </c>
       <c r="D2">
-        <v>48.52</v>
+        <v>76.20999999999999</v>
       </c>
       <c r="E2">
         <v>513</v>
@@ -428,13 +428,13 @@
         <v>1000</v>
       </c>
       <c r="B3">
-        <v>8.52</v>
+        <v>8.81</v>
       </c>
       <c r="C3">
-        <v>4.554</v>
+        <v>8.465999999999999</v>
       </c>
       <c r="D3">
-        <v>49.68</v>
+        <v>78.15000000000001</v>
       </c>
       <c r="E3">
         <v>513</v>
@@ -445,13 +445,13 @@
         <v>2000</v>
       </c>
       <c r="B4">
-        <v>12.4</v>
+        <v>12.65</v>
       </c>
       <c r="C4">
-        <v>4.564</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="D4">
-        <v>50.78</v>
+        <v>80.06999999999999</v>
       </c>
       <c r="E4">
         <v>513</v>
@@ -462,13 +462,13 @@
         <v>5000</v>
       </c>
       <c r="B5">
-        <v>23.52</v>
+        <v>23.74</v>
       </c>
       <c r="C5">
-        <v>4.601</v>
+        <v>8.821</v>
       </c>
       <c r="D5">
-        <v>51.86</v>
+        <v>82.18000000000001</v>
       </c>
       <c r="E5">
         <v>513</v>
@@ -479,13 +479,13 @@
         <v>10000</v>
       </c>
       <c r="B6">
-        <v>41.5</v>
+        <v>41.7</v>
       </c>
       <c r="C6">
-        <v>4.642</v>
+        <v>8.965999999999999</v>
       </c>
       <c r="D6">
-        <v>52.35</v>
+        <v>83.33</v>
       </c>
       <c r="E6">
         <v>513</v>
@@ -496,13 +496,13 @@
         <v>20000</v>
       </c>
       <c r="B7">
-        <v>76.84999999999999</v>
+        <v>77.03</v>
       </c>
       <c r="C7">
-        <v>4.658</v>
+        <v>8.99</v>
       </c>
       <c r="D7">
-        <v>65.55</v>
+        <v>84.12</v>
       </c>
       <c r="E7">
         <v>513</v>

</xml_diff>